<commit_message>
changed model to qwen2.5-Q4_K_S
</commit_message>
<xml_diff>
--- a/res/efficiency/pet-md/ultiima-32b-Q4_K_S/2025-02-12_15-01-27/efficiency.xlsx
+++ b/res/efficiency/pet-md/ultiima-32b-Q4_K_S/2025-02-12_15-01-27/efficiency.xlsx
@@ -1,36 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felix\Documents\llm-process-generation\res\efficiency\pet-md\ultiima-32b-Q4_K_S\2025-02-12_15-01-27\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72C03B89-B244-4961-8C36-6434517C33BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Power_Stats" sheetId="1" r:id="rId1"/>
     <sheet name="Answer_Stats" sheetId="2" r:id="rId2"/>
     <sheet name="Error_Stats" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -109,8 +90,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -169,25 +150,17 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -225,7 +198,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -259,7 +232,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -294,10 +266,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -470,16 +441,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.5546875" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -490,7 +456,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -507,15 +473,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="14.109375" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -532,7 +494,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -549,7 +511,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -572,15 +534,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -588,7 +546,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>21</v>
       </c>

</xml_diff>